<commit_message>
Blankett 1.10 (referenskopia): karteringsstatus enligt metodik R3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018dW3eVThxZy88p962tyuWT
</commit_message>
<xml_diff>
--- a/blanketter/blankett_forvaltarkunskap_nnk.xlsx
+++ b/blanketter/blankett_forvaltarkunskap_nnk.xlsx
@@ -741,7 +741,7 @@
     <row r="3" ht="15" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Länsstyrelsen i Södermanlands län · Naturskyddsenheten · NNK/NRF ref. 2451-2026 · version 1.8, 2026-08-27</t>
+          <t>Länsstyrelsen i Södermanlands län · Naturskyddsenheten · NNK/NRF ref. 2451-2026 · version 1.10, 2026-10-19</t>
         </is>
       </c>
     </row>
@@ -45996,7 +45996,7 @@
       </c>
       <c r="E19" s="27" t="inlineStr">
         <is>
-          <t>2 Granskad vid skrivbordet för förvaltarkunskap och dokument. 3 Besökt i fält om förvaltaren faktiskt varit där nyligen. 4 Inventerad i fält endast vid standardiserad metodik.</t>
+          <t>2 Granskad vid skrivbordet för förvaltarkunskap och dokument. 3 Besökt i fält om förvaltaren faktiskt varit där nyligen. 4 Inventerad i fält bara om ytan själv är inventerad med NV:s metod för basinventering eller uppföljning; TUVA och andra lånade inventeringar ger 2.</t>
         </is>
       </c>
     </row>

</xml_diff>